<commit_message>
Adding new assets, completing the rooms
</commit_message>
<xml_diff>
--- a/Docs/asset-references.xlsx
+++ b/Docs/asset-references.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Games\UnderTheSofa\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{460E44C3-04FF-4A96-86B7-3B070221B749}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20C54E38-4A8E-4533-8EC1-3B2E1C0F77E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8340" yWindow="1080" windowWidth="28800" windowHeight="15345" xr2:uid="{75B83A5A-1663-41E6-AA10-87552D6FB11F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{75B83A5A-1663-41E6-AA10-87552D6FB11F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,41 +39,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="32">
   <si>
     <t>asset links</t>
   </si>
   <si>
-    <t>cars</t>
-  </si>
-  <si>
-    <t>https://ggbot.itch.io/psx-style-cars</t>
-  </si>
-  <si>
-    <t>vegetat</t>
-  </si>
-  <si>
-    <t>https://itch.io/queue/c/6139762/non-kenney-quaternius-or-kaykit-lo-fi-cc0-3d-game-assets?game_id=4920619&amp;password=</t>
-  </si>
-  <si>
-    <t>retro urban kit</t>
-  </si>
-  <si>
-    <t>https://kenney-assets.itch.io/retro-urban-kit</t>
-  </si>
-  <si>
-    <t>retro modular house</t>
-  </si>
-  <si>
-    <t>https://elegantcrow.itch.io/retro-modular-house-pack</t>
-  </si>
-  <si>
-    <t>buildings urban</t>
-  </si>
-  <si>
-    <t>https://valsekamerplant.itch.io/psx-style-urban-stacked-pack</t>
-  </si>
-  <si>
     <t>office things</t>
   </si>
   <si>
@@ -86,54 +56,15 @@
     <t>https://rohhsa.itch.io/free-psx-ui</t>
   </si>
   <si>
-    <t>https://valsekamerplant.itch.io/psx-style-house-plants-and-pots</t>
-  </si>
-  <si>
-    <t>pots and plants</t>
-  </si>
-  <si>
-    <t>https://nicowlas.itch.io/psx-kitchen-props-pack</t>
-  </si>
-  <si>
-    <t>kitchen</t>
-  </si>
-  <si>
-    <t>https://craigsnedeker.itch.io/classic64-asset-library</t>
-  </si>
-  <si>
-    <t>random assets</t>
-  </si>
-  <si>
-    <t>house 3d model</t>
-  </si>
-  <si>
     <t>https://mcpato.itch.io/house-interior-psx-assets</t>
   </si>
   <si>
-    <t>https://sketchfab.com/3d-models/table-top-racing-firefly-bbq-2fc12d167b8848ce8f1c8a02ee13b6d7</t>
-  </si>
-  <si>
-    <t>tabletop racing</t>
-  </si>
-  <si>
-    <t>https://sketchfab.com/3d-models/table-top-racing-beach-buggies-b159fb5373bc46edb6fb291f6d238f3f</t>
-  </si>
-  <si>
-    <t>https://sketchfab.com/3d-models/table-top-racing-rusty-nuts-workshop-8ac8eef11e404195985dee59dabd5eb7</t>
-  </si>
-  <si>
-    <t>garaza stol za trkanje</t>
-  </si>
-  <si>
     <t>https://sketchfab.com/3d-models/table-top-racing-toys-r-asleep-5e6fca61cc5e4d85a20675fd141b97b1</t>
   </si>
   <si>
     <t>spavaca stol za trkanje</t>
   </si>
   <si>
-    <t>bolji stol vanjski za trkanje</t>
-  </si>
-  <si>
     <t>https://sketchfab.com/3d-models/lamborghini-countach-ccbd31682fb64ce9979b7376a7658417</t>
   </si>
   <si>
@@ -167,13 +98,43 @@
     <t>https://sketchfab.com/3d-models/2001-acura-integra-type-r-343a13e17f544a788b9b02fbfc6c58b7</t>
   </si>
   <si>
-    <t>2001 Acura Integra Type-R</t>
-  </si>
-  <si>
-    <t>table top racing - nighttime noodles</t>
-  </si>
-  <si>
-    <t>https://sketchfab.com/3d-models/table-top-racing-nighttime-noodles-1f8a8a8856cd4f2a95ef29cac4c9f9b7</t>
+    <t>https://sketchfab.com/3d-models/simple-golden-ring-b3f29a75a90445e59b5f0c2ec6bd6ecf#download</t>
+  </si>
+  <si>
+    <t>https://fabledindiagames.itch.io/psxmodels</t>
+  </si>
+  <si>
+    <t>https://assetstore.unity.com/packages/audio/sound-fx/doors-small-sound-pack-262071</t>
+  </si>
+  <si>
+    <t>Door sound effects</t>
+  </si>
+  <si>
+    <t>Bathroom assets</t>
+  </si>
+  <si>
+    <t>https://assetstore.unity.com/packages/3d/props/furniture/bathroom-set-interior-263462</t>
+  </si>
+  <si>
+    <t>https://sketchfab.com/3d-models/bathroom-props-set-low-poly-5b4781c82c4e4b67a44323473da5f37d</t>
+  </si>
+  <si>
+    <t>Living room dresser</t>
+  </si>
+  <si>
+    <t>https://assetstore.unity.com/packages/3d/props/furniture/furniture-mega-pack-free-330002</t>
+  </si>
+  <si>
+    <t>Match boxes and rice balls - kitchen deco</t>
+  </si>
+  <si>
+    <t>2001 Acura Integra Type-R - player model</t>
+  </si>
+  <si>
+    <t>Gold rings</t>
+  </si>
+  <si>
+    <t>House model</t>
   </si>
 </sst>
 </file>
@@ -197,12 +158,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -218,9 +185,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -556,10 +525,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{886A93FD-C5CA-4B9A-AFFE-847FB8953B63}">
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="36.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="38.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="112" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -569,7 +538,7 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -585,19 +554,19 @@
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="A4" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" t="s">
         <v>5</v>
       </c>
-      <c r="B4" t="s">
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" t="s">
         <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -605,28 +574,28 @@
         <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" t="s">
         <v>11</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="B8" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B9" t="s">
         <v>15</v>
@@ -634,124 +603,73 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B10" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="A11" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" t="s">
         <v>20</v>
       </c>
-      <c r="B11" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" t="s">
         <v>21</v>
       </c>
-      <c r="B12" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="1" t="s">
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>30</v>
-      </c>
-      <c r="B14" t="s">
+      <c r="B16" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" t="s">
         <v>27</v>
-      </c>
-      <c r="B15" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>29</v>
-      </c>
-      <c r="B16" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>32</v>
-      </c>
-      <c r="B17" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>33</v>
-      </c>
-      <c r="B18" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>35</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>37</v>
-      </c>
-      <c r="B20" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>39</v>
-      </c>
-      <c r="B21" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>42</v>
-      </c>
-      <c r="B22" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>43</v>
-      </c>
-      <c r="B23" t="s">
-        <v>44</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" xr:uid="{CDB0DFEA-64DD-496A-B83D-6A0555EA444B}"/>
-    <hyperlink ref="B3" r:id="rId2" xr:uid="{B676653A-FCF8-42D8-8A84-0FDE0A48D43F}"/>
-    <hyperlink ref="B5" r:id="rId3" xr:uid="{EF4434B0-6F2A-448F-922E-4FF2BC74ED8E}"/>
-    <hyperlink ref="B7" r:id="rId4" xr:uid="{0D260C26-F4C1-49A0-8EBC-F07A42CDB40B}"/>
-    <hyperlink ref="B19" r:id="rId5" xr:uid="{610D823A-90A7-47CF-BE71-5D05357B3170}"/>
-    <hyperlink ref="B13" r:id="rId6" xr:uid="{E84DA550-BB10-40C1-8356-32A51680E1B1}"/>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{0D260C26-F4C1-49A0-8EBC-F07A42CDB40B}"/>
+    <hyperlink ref="B8" r:id="rId2" xr:uid="{610D823A-90A7-47CF-BE71-5D05357B3170}"/>
+    <hyperlink ref="B3" r:id="rId3" xr:uid="{FA37FD59-02D1-44F8-B543-7D48E701DA85}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
improving visuals, ambient lighting, adding particles and sound effects
</commit_message>
<xml_diff>
--- a/Docs/asset-references.xlsx
+++ b/Docs/asset-references.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Games\UnderTheSofa\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20C54E38-4A8E-4533-8EC1-3B2E1C0F77E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1D2D7DD-092A-439F-A0D1-87091D381BE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{75B83A5A-1663-41E6-AA10-87552D6FB11F}"/>
+    <workbookView xWindow="8340" yWindow="1080" windowWidth="28800" windowHeight="15345" xr2:uid="{75B83A5A-1663-41E6-AA10-87552D6FB11F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -189,7 +189,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -546,10 +546,10 @@
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="3" t="s">
         <v>4</v>
       </c>
     </row>
@@ -562,7 +562,7 @@
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="A5" t="s">
         <v>7</v>
       </c>
       <c r="B5" t="s">

</xml_diff>

<commit_message>
adding music tracks and UI tweaks
</commit_message>
<xml_diff>
--- a/Docs/asset-references.xlsx
+++ b/Docs/asset-references.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Games\UnderTheSofa\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1D2D7DD-092A-439F-A0D1-87091D381BE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FDA2C89-92C3-4DEA-99A8-A2AC28A839BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8340" yWindow="1080" windowWidth="28800" windowHeight="15345" xr2:uid="{75B83A5A-1663-41E6-AA10-87552D6FB11F}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="34">
   <si>
     <t>asset links</t>
   </si>
@@ -135,6 +135,12 @@
   </si>
   <si>
     <t>House model</t>
+  </si>
+  <si>
+    <t>Collectibles sound effects</t>
+  </si>
+  <si>
+    <t>https://pixabay.com/sound-effects/film-special-effects-money-pickup-2-89563/</t>
   </si>
 </sst>
 </file>
@@ -525,7 +531,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{886A93FD-C5CA-4B9A-AFFE-847FB8953B63}">
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="38.140625" bestFit="1" customWidth="1"/>
@@ -665,11 +671,20 @@
         <v>27</v>
       </c>
     </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" xr:uid="{0D260C26-F4C1-49A0-8EBC-F07A42CDB40B}"/>
     <hyperlink ref="B8" r:id="rId2" xr:uid="{610D823A-90A7-47CF-BE71-5D05357B3170}"/>
     <hyperlink ref="B3" r:id="rId3" xr:uid="{FA37FD59-02D1-44F8-B543-7D48E701DA85}"/>
+    <hyperlink ref="B18" r:id="rId4" xr:uid="{6BDE16DF-0410-46F4-B402-A69EA0A63531}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>